<commit_message>
Add new product images and update sourcing manifest
</commit_message>
<xml_diff>
--- a/SkinVault_Image_Sourcing_Manifest.xlsx
+++ b/SkinVault_Image_Sourcing_Manifest.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Image Sourcing" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Image Sourcing" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -829,7 +829,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Page sourced</t>
+          <t>Downloaded</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Page sourced</t>
+          <t>Downloaded</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Page sourced</t>
+          <t>Downloaded</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Page sourced</t>
+          <t>Downloaded</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Page sourced</t>
+          <t>Downloaded</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Page sourced</t>
+          <t>Downloaded</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H120" s="4" t="inlineStr">
         <is>
-          <t>Page sourced</t>
+          <t>Downloaded</t>
         </is>
       </c>
       <c r="I120" s="7" t="inlineStr">

</xml_diff>